<commit_message>
broad changes to esco ds class (now occ framework). changes regarding aggregation of esco data to isco level. evaluation of the distribution of GBN shares by isco group. distribution visible in industry, occupation and regional plots is coherent with that. so what needs to be improved is the underlying data! evaluation of problems with onet-esco crosswalk.
</commit_message>
<xml_diff>
--- a/results/validation/onet_esco_crosswalk/onet_to_esco_match_summary.xlsx
+++ b/results/validation/onet_esco_crosswalk/onet_to_esco_match_summary.xlsx
@@ -1,14 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\gess-fs.d.ethz.ch\home$\fzaussinger\Documents\Projects\04_jrc_green-skills-regional\03_data-analysis\re4gt\results\validation\onet_esco_crosswalk\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="T:\Documents\Projects\04_jrc_green-skills-regional\03_data-analysis\re4gt\results\validation\onet_esco_crosswalk\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:40009_{D8D552BF-6DB1-4FA0-B48D-8AD66FC8074C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="-16320" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
@@ -1418,7 +1417,6 @@
         <sz val="11"/>
         <color theme="1"/>
         <name val="Calibri"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </font>
     </dxf>
@@ -1438,7 +1436,7 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:E139" totalsRowShown="0" headerRowDxfId="0">
   <autoFilter ref="A1:E139"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E139">
+  <sortState ref="A2:E139">
     <sortCondition descending="1" ref="E1:E139"/>
   </sortState>
   <tableColumns count="5">
@@ -1750,16 +1748,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E139"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.90625" customWidth="1"/>
-    <col min="2" max="2" width="83.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.08984375" customWidth="1"/>
-    <col min="5" max="5" width="16.81640625" customWidth="1"/>
+    <col min="1" max="1" width="11.85546875" customWidth="1"/>
+    <col min="2" max="2" width="83.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.140625" customWidth="1"/>
+    <col min="5" max="5" width="16.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1776,7 +1774,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1793,7 +1791,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1810,7 +1808,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -1827,7 +1825,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -1844,7 +1842,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -1861,7 +1859,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -1878,7 +1876,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>18</v>
       </c>
@@ -1895,7 +1893,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -1912,7 +1910,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -1929,7 +1927,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>24</v>
       </c>
@@ -1946,7 +1944,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>26</v>
       </c>
@@ -1963,7 +1961,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>28</v>
       </c>
@@ -1980,7 +1978,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>30</v>
       </c>
@@ -1997,7 +1995,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>33</v>
       </c>
@@ -2014,7 +2012,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>35</v>
       </c>
@@ -2031,7 +2029,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>37</v>
       </c>
@@ -2048,7 +2046,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>39</v>
       </c>
@@ -2065,7 +2063,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>41</v>
       </c>
@@ -2082,7 +2080,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>43</v>
       </c>
@@ -2099,7 +2097,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>45</v>
       </c>
@@ -2116,7 +2114,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>47</v>
       </c>
@@ -2133,7 +2131,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>49</v>
       </c>
@@ -2150,7 +2148,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>51</v>
       </c>
@@ -2167,7 +2165,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>53</v>
       </c>
@@ -2184,7 +2182,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>55</v>
       </c>
@@ -2201,7 +2199,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>57</v>
       </c>
@@ -2218,7 +2216,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>59</v>
       </c>
@@ -2235,7 +2233,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>61</v>
       </c>
@@ -2252,7 +2250,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>63</v>
       </c>
@@ -2269,7 +2267,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>65</v>
       </c>
@@ -2286,7 +2284,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>67</v>
       </c>
@@ -2303,7 +2301,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>69</v>
       </c>
@@ -2320,7 +2318,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>71</v>
       </c>
@@ -2337,7 +2335,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>73</v>
       </c>
@@ -2354,7 +2352,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>75</v>
       </c>
@@ -2371,7 +2369,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>77</v>
       </c>
@@ -2388,7 +2386,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>79</v>
       </c>
@@ -2405,7 +2403,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>81</v>
       </c>
@@ -2422,7 +2420,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>83</v>
       </c>
@@ -2439,7 +2437,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>85</v>
       </c>
@@ -2456,7 +2454,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>87</v>
       </c>
@@ -2473,7 +2471,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>89</v>
       </c>
@@ -2490,7 +2488,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>91</v>
       </c>
@@ -2507,7 +2505,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>93</v>
       </c>
@@ -2524,7 +2522,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>95</v>
       </c>
@@ -2541,7 +2539,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>97</v>
       </c>
@@ -2558,7 +2556,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>100</v>
       </c>
@@ -2575,7 +2573,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>102</v>
       </c>
@@ -2592,7 +2590,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>104</v>
       </c>
@@ -2609,7 +2607,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>106</v>
       </c>
@@ -2626,7 +2624,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>108</v>
       </c>
@@ -2643,7 +2641,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>110</v>
       </c>
@@ -2660,7 +2658,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>112</v>
       </c>
@@ -2677,7 +2675,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>114</v>
       </c>
@@ -2694,7 +2692,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>116</v>
       </c>
@@ -2711,7 +2709,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>118</v>
       </c>
@@ -2728,7 +2726,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>120</v>
       </c>
@@ -2745,7 +2743,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>122</v>
       </c>
@@ -2762,7 +2760,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>124</v>
       </c>
@@ -2779,7 +2777,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>126</v>
       </c>
@@ -2796,7 +2794,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>128</v>
       </c>
@@ -2813,7 +2811,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>130</v>
       </c>
@@ -2830,7 +2828,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>132</v>
       </c>
@@ -2847,7 +2845,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>134</v>
       </c>
@@ -2864,7 +2862,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>136</v>
       </c>
@@ -2881,7 +2879,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>138</v>
       </c>
@@ -2898,7 +2896,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>140</v>
       </c>
@@ -2915,7 +2913,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>142</v>
       </c>
@@ -2932,7 +2930,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>144</v>
       </c>
@@ -2949,7 +2947,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>146</v>
       </c>
@@ -2966,7 +2964,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>148</v>
       </c>
@@ -2983,7 +2981,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>150</v>
       </c>
@@ -3000,7 +2998,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>152</v>
       </c>
@@ -3017,7 +3015,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>154</v>
       </c>
@@ -3034,7 +3032,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>156</v>
       </c>
@@ -3051,7 +3049,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>158</v>
       </c>
@@ -3068,7 +3066,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>160</v>
       </c>
@@ -3085,7 +3083,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>162</v>
       </c>
@@ -3102,7 +3100,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>164</v>
       </c>
@@ -3119,7 +3117,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>166</v>
       </c>
@@ -3136,7 +3134,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>168</v>
       </c>
@@ -3153,7 +3151,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>170</v>
       </c>
@@ -3170,7 +3168,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>172</v>
       </c>
@@ -3187,7 +3185,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>174</v>
       </c>
@@ -3204,7 +3202,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>176</v>
       </c>
@@ -3221,7 +3219,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>178</v>
       </c>
@@ -3238,7 +3236,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>180</v>
       </c>
@@ -3255,7 +3253,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>182</v>
       </c>
@@ -3272,7 +3270,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>184</v>
       </c>
@@ -3289,7 +3287,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>186</v>
       </c>
@@ -3306,7 +3304,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>188</v>
       </c>
@@ -3323,7 +3321,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>190</v>
       </c>
@@ -3340,7 +3338,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>192</v>
       </c>
@@ -3357,7 +3355,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>194</v>
       </c>
@@ -3374,7 +3372,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>196</v>
       </c>
@@ -3391,7 +3389,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>198</v>
       </c>
@@ -3408,7 +3406,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>200</v>
       </c>
@@ -3425,7 +3423,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>202</v>
       </c>
@@ -3442,7 +3440,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>204</v>
       </c>
@@ -3459,7 +3457,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>206</v>
       </c>
@@ -3476,7 +3474,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>208</v>
       </c>
@@ -3493,7 +3491,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>210</v>
       </c>
@@ -3510,7 +3508,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>212</v>
       </c>
@@ -3527,7 +3525,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>214</v>
       </c>
@@ -3544,7 +3542,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>216</v>
       </c>
@@ -3561,7 +3559,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>218</v>
       </c>
@@ -3578,7 +3576,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>220</v>
       </c>
@@ -3595,7 +3593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>222</v>
       </c>
@@ -3612,7 +3610,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>224</v>
       </c>
@@ -3629,7 +3627,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>226</v>
       </c>
@@ -3646,7 +3644,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>228</v>
       </c>
@@ -3663,7 +3661,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>230</v>
       </c>
@@ -3680,7 +3678,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>232</v>
       </c>
@@ -3697,7 +3695,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>234</v>
       </c>
@@ -3714,7 +3712,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>236</v>
       </c>
@@ -3731,7 +3729,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>238</v>
       </c>
@@ -3748,7 +3746,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>240</v>
       </c>
@@ -3765,7 +3763,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>242</v>
       </c>
@@ -3782,7 +3780,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>244</v>
       </c>
@@ -3799,7 +3797,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>246</v>
       </c>
@@ -3816,7 +3814,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>248</v>
       </c>
@@ -3833,7 +3831,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>250</v>
       </c>
@@ -3850,7 +3848,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>252</v>
       </c>
@@ -3867,7 +3865,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>254</v>
       </c>
@@ -3884,7 +3882,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>256</v>
       </c>
@@ -3901,7 +3899,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>258</v>
       </c>
@@ -3918,7 +3916,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>260</v>
       </c>
@@ -3935,7 +3933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>262</v>
       </c>
@@ -3952,7 +3950,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>264</v>
       </c>
@@ -3969,7 +3967,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>266</v>
       </c>
@@ -3986,7 +3984,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>268</v>
       </c>
@@ -4003,7 +4001,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>270</v>
       </c>
@@ -4020,7 +4018,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>272</v>
       </c>
@@ -4037,7 +4035,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>274</v>
       </c>
@@ -4054,7 +4052,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>276</v>
       </c>
@@ -4071,7 +4069,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>278</v>
       </c>
@@ -4088,7 +4086,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>280</v>
       </c>
@@ -4105,7 +4103,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>282</v>
       </c>

</xml_diff>